<commit_message>
Fill HSK2 parts 1 (ID 501-550) with parts of speech
</commit_message>
<xml_diff>
--- a/HSK2_parts_of_speech_1(501-550).xlsx
+++ b/HSK2_parts_of_speech_1(501-550).xlsx
@@ -644,6 +644,16 @@
           <t>фразовая частица восклицательных и побудительных предложений</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>частица-восклицание «а!» (также междометие при удивлении)</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (служебное слово)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -670,6 +680,16 @@
           <t>чувство любви</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>любовь (чувство)</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>отвлечённое существительное</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -696,6 +716,16 @@
           <t>возлюбленный, возлюбленная</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>супруг / супруга</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>существительное; в КНР — вежливое обозначение мужа/жены</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -722,6 +752,11 @@
           <t>спокойный, тихий</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>спокойный, тихий</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -748,6 +783,16 @@
           <t>безопасность; безопасный</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>безопасность</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>безопасный</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -774,6 +819,21 @@
           <t>белый цвет</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>белый цвет</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>белый (атрибутивное цветовое слово, требует 的 перед существительным)</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>цветовые слова с 色 образуют пару: 白 — прилагательное, 白色 — существительное/区分词</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -800,6 +860,11 @@
           <t>староста группы</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>староста (группы, класса)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -826,6 +891,16 @@
           <t>полночь; полночи</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>полночь; глубокая ночь</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>полночный (атрибутив: 半夜的电话)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -852,6 +927,11 @@
           <t>выполнять, делать</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>делать, заниматься, устраивать (办事, 办学校)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -878,6 +958,11 @@
           <t>способ, метод</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>способ, метод, выход (想个办法)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -904,6 +989,11 @@
           <t>офис</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>офис, служебный кабинет</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -930,6 +1020,21 @@
           <t>помогать; помощь</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>помощь</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>помогать</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>离合词: 帮助了他很多忙</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -956,6 +1061,16 @@
           <t>полный</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>обнимать, держать на руках (抱孩子)</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>в значении «полный» из эталона — редкое/книжное, основное значение — глагол</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -982,6 +1097,16 @@
           <t>зарегистрироваться</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>записываться, подавать заявку (报名学习)</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>离合词: 报过名, 报个名</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1008,6 +1133,16 @@
           <t>газета</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>газета</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>для газетных экземпляров (一张报纸 — но счётное 张; само 报纸 — нет)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1034,6 +1169,16 @@
           <t>север</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>север, северная сторона</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>северный (北方的天气)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1060,6 +1205,16 @@
           <t>заучивать</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>заучивать наизусть (背课文)</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>многозначно: bèi — спина (сущ.), bēi — нести на спине (глаг.)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1086,6 +1241,16 @@
           <t>например, допустим</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>например, допустим (引入 пример)</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>служебное слово-союз</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1112,6 +1277,16 @@
           <t>например</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>например (разговорный вариант 比如)</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>устойчивое выражение-конструкция (比如 + предложение)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1138,6 +1313,16 @@
           <t>ручка</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ручка, кисть (写毛笔字)</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>письменные принадлежности считаются словом 支, а не 笔; 笔 как счётное — для денежных сумм (一笔钱)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1164,6 +1349,21 @@
           <t>записывать; заметки</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>конспект, записи</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>вести записи</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>笔记本/笔记本 — другое слово</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1190,6 +1390,11 @@
           <t>блокнот</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>блокнот; ноутбук (笔记本电脑)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1216,6 +1421,11 @@
           <t>обязательно следует</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>обязательно, необходимо (должно + глагол)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1242,6 +1452,16 @@
           <t>сторона</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>край, сторона, граница (河边)</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>суффикс локатива после слов (上边, 外边)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1268,6 +1488,11 @@
           <t>меняться</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>меняться, становиться другим (变了)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1294,6 +1519,16 @@
           <t>превратиться в..., измениться в...</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>превращаться в..., измениться в...</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>глагол + результативное дополнение 成 (离合: 变成了...</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1320,6 +1555,11 @@
           <t>раз (счётное слово для действий)</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>раз (счётное для повторений действия: 看一遍, 说三遍)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1346,6 +1586,16 @@
           <t>часы</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>часы (手表); таблица, график (时间表); поверхность (表面)</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>выражать, давать понять (表示同义误用)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1372,6 +1622,11 @@
           <t>выражать</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>показывать, выражать, означать (这表示什么?)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1398,6 +1653,11 @@
           <t>неплохо, хорошо</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>неплохо, хорошо (身体不错)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1424,6 +1684,21 @@
           <t>не только</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>даже не (他不但没来)</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>не только (不但……而且…)</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>коррелятивная конструкция союзов</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1450,6 +1725,21 @@
           <t>недостаточно</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>недостаточно, не хватать (钱不够)</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>недостаточный (水平不够)</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>отрицательная форма от 够</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1476,6 +1766,21 @@
           <t>тем не менее</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>только лишь, всего (不过三个人)</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>однако, тем не менее (межчастное соединение предложений)</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>две функции: союз и ограничительно-числительное наречие</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1502,6 +1807,16 @@
           <t>не слишком</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>не слишком (不太好吃)</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>грамматическая конструкция: отрицание 不 + наречие 太 + прилагательное</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1528,6 +1843,21 @@
           <t>не (категорическое запрещение)</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>не хотеть ( obsolete )</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>не надо, не следует (不要抽烟)</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>категорическое запрещение/отказ; конструкция 不 + 要</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1554,6 +1884,16 @@
           <t>извините; неловко</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>неловко, совестно; извините</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>устойчивое выражение (вежливая формула), разнимается: 很不好意思</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1580,6 +1920,21 @@
           <t>скоро</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>некоторое время (不久以后)</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>вскоре, незадолго (他不久就来了)</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>отрицание 不 + 久</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1606,6 +1961,21 @@
           <t>недовольный</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>недовольство</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>не удовлетворять (不满十人)</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>недовольный (他对我不满)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1632,6 +2002,21 @@
           <t>уступать, хуже</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>уступать, быть хуже (A不如B)</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>не лучше, чем (与其…不如…)</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>конструкция сравнения</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1658,6 +2043,21 @@
           <t>немало, достаточно много</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>немало, довольно много (不少人)</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>изрядно (等了不少时间)</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>литота: 不 + 少</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1684,6 +2084,26 @@
           <t>разный</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>различие, отличие (有很大不同)</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>не одинаково, отличается (两人不同)</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>различный, отличающийся (不同的国家)</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>отрицание 不 + 同</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1710,6 +2130,21 @@
           <t>нельзя, не годится</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>не сможет, не пройдёт (时间不行)</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>нельзя, не годится, не подходит (这样不行)</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>отрицание 不 + 行</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1736,6 +2171,16 @@
           <t>необязательно</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>не обязательно, навряд ли (不一定来)</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>отрицание 不 + 一定</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1762,6 +2207,16 @@
           <t>скоро</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>через мгновение, вскоре (不一会儿他就回来了)</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>устойчивая временная конструкция (不 + 一会儿)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1788,6 +2243,16 @@
           <t>часть</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>часть, доля (一部分, 两部分)</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>для частей (分为三部分)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1814,6 +2279,21 @@
           <t>только</t>
         </is>
       </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>возраст «всего…» (他今年才二十岁)</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>только тогда, лишь, недавно (才来, 才知道)</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>сложное наречие; подчёркивает запоздалость/условность (你走了我才说) — одно из труднейших слов</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1840,6 +2320,11 @@
           <t>меню</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>меню, карточка блюд</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1866,6 +2351,16 @@
           <t>посещать</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>посещать, осматривать (参观工厂)</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>离合词: 参观了一下</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1892,6 +2387,16 @@
           <t>участвовать</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>принимать участие, участвовать (参加比赛)</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>离合词: 参加了一次</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1916,6 +2421,11 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>трава</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>трава; черновик (草稿)</t>
         </is>
       </c>
     </row>

</xml_diff>